<commit_message>
Update stock radar data and reports
</commit_message>
<xml_diff>
--- a/output/radar_latest.xlsx
+++ b/output/radar_latest.xlsx
@@ -14,7 +14,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'技術雷達'!$A$1:$A$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'覆蓋率'!$A$1:$J$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'資料擷取紀錄'!$A$1:$F$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'資料擷取紀錄'!$A$1:$F$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -542,7 +542,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-11T00:05:32.073894+08:00</t>
+          <t>2026-10-11T00:13:32.082833+08:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1980</v>
+        <v>1982</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -593,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -662,7 +662,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-10-10 16:04:33</t>
+          <t>2026-10-10 16:09:58</t>
         </is>
       </c>
     </row>
@@ -692,7 +692,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-10-10 16:04:28</t>
+          <t>2026-10-10 16:09:56</t>
         </is>
       </c>
     </row>
@@ -1060,8 +1060,1532 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>868</v>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:10:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1084</v>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:10:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>empty_unverified</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>No rows; holiday or schema drift</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:10:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>empty_unverified</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>No rows; holiday or schema drift</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:10:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>empty_unverified</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>No rows; holiday or schema drift</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:10:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>empty_unverified</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>No rows; holiday or schema drift</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:10:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>870</v>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:10:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1079</v>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:10:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>868</v>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:10:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1082</v>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:10:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>872</v>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:10:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1084</v>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:10:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>875</v>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:10:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>1085</v>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:10:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>868</v>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:10:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1081</v>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:10:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>867</v>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:11:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1081</v>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:10:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>874</v>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:11:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>1075</v>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:11:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>868</v>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:11:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1080</v>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:11:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>866</v>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:11:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:11:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>862</v>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:11:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>1082</v>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:11:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>860</v>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:11:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>1081</v>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:11:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>867</v>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:11:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>1087</v>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:11:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>866</v>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:11:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>1084</v>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:11:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>875</v>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>1087</v>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:11:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>861</v>
+      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:12:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>1083</v>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:12:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>864</v>
+      </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:12:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:12:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>857</v>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:12:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>1084</v>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:12:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>865</v>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:12:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>1081</v>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:12:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>859</v>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:12:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>1084</v>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:12:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>872</v>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:12:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>1083</v>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:12:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>868</v>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:12:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>1084</v>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:12:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>872</v>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:12:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>1085</v>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:12:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>861</v>
+      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:13:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>1082</v>
+      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:13:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>860</v>
+      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:13:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>1084</v>
+      </c>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:13:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>878</v>
+      </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:13:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>1079</v>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:13:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>TPEX</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>867</v>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:13:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>TWSE</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>1083</v>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:13:24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F17"/>
+  <autoFilter ref="A1:F75"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>